<commit_message>
Corte publicado desde el tablero · 12/9/2026, 8:19:21 a.m.
</commit_message>
<xml_diff>
--- a/datos/Control_Plantillas_NetSuite_V1.xlsx
+++ b/datos/Control_Plantillas_NetSuite_V1.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Control_Plantillas" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Control_Plantillas!$A$3:$AE$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Control_Plantillas!$A$3:$AE$44</definedName>
     <definedName name="Cat_Areas">Catalogos!$H$3:$H$10</definedName>
     <definedName name="Cat_Estatus">Catalogos!$A$3:$A$7</definedName>
     <definedName name="Cat_Etapas">Catalogos!$J$3:$J$8</definedName>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="759" uniqueCount="285">
   <si>
     <t>CATÁLOGOS - No modificar sin autorización del PMO</t>
   </si>
@@ -812,18 +812,6 @@
   </si>
   <si>
     <t>2026-06-04</t>
-  </si>
-  <si>
-    <t>MFG-02</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>Artículos Otros Cargos para la Compra</t>
-  </si>
-  <si>
-    <t>2026-05-19</t>
   </si>
   <si>
     <t>MFG-03</t>
@@ -1270,7 +1258,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="10">
     <dxf>
       <font>
         <b/>
@@ -1282,20 +1270,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFE4E7EC"/>
           <bgColor rgb="FFE4E7EC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1364,226 +1338,6 @@
       </font>
       <fill>
         <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-        <color rgb="FF667085"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E7EC"/>
-          <bgColor rgb="FFE4E7EC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C6500"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF006100"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-        <color rgb="FF667085"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E7EC"/>
-          <bgColor rgb="FFE4E7EC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C6500"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF006100"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-        <color rgb="FF667085"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E7EC"/>
-          <bgColor rgb="FFE4E7EC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C6500"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF006100"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="9"/>
-        <color rgb="FF667085"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE4E7EC"/>
-          <bgColor rgb="FFE4E7EC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF9C6500"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FF006100"/>
-        <name val="Arial"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -1903,8 +1657,8 @@
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="12">
-        <f>COUNTA(Control_Plantillas!$A$4:$A$60)</f>
-        <v>43</v>
+        <f>COUNTA(Control_Plantillas!$A$4:$A$59)</f>
+        <v>42</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>56</v>
@@ -1937,18 +1691,18 @@
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="14">
-        <f>IFERROR(AVERAGE(Control_Plantillas!$Z$4:$Z$60),0)</f>
-        <v>0.27674418604651135</v>
+        <f>IFERROR(AVERAGE(Control_Plantillas!$Z$4:$Z$59),0)</f>
+        <v>0.2785714285714283</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="17">
-        <f>COUNTIF(Control_Plantillas!$B$4:$B$60,$E7)</f>
+        <f>COUNTIF(Control_Plantillas!$B$4:$B$59,$E7)</f>
         <v>6</v>
       </c>
       <c r="G7" s="18">
-        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$60,$E7,Control_Plantillas!$Z$4:$Z$60),0)</f>
+        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$59,$E7,Control_Plantillas!$Z$4:$Z$59),0)</f>
         <v>0.65833333333333333</v>
       </c>
       <c r="H7" s="17">
@@ -1958,15 +1712,15 @@
         <v>6</v>
       </c>
       <c r="J7" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E7,Control_Plantillas!$O$4:$O$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E7,Control_Plantillas!$O$4:$O$59,"Completado")</f>
         <v>5</v>
       </c>
       <c r="K7" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E7,Control_Plantillas!$R$4:$R$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E7,Control_Plantillas!$R$4:$R$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="L7" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E7,Control_Plantillas!$U$4:$U$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E7,Control_Plantillas!$U$4:$U$59,"Completado")</f>
         <v>0</v>
       </c>
     </row>
@@ -1976,38 +1730,38 @@
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="12">
-        <f>COUNTIF(Control_Plantillas!$I$4:$I$60,"Completado")</f>
+        <f>COUNTIF(Control_Plantillas!$I$4:$I$59,"Completado")</f>
         <v>8</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="17">
-        <f>COUNTIF(Control_Plantillas!$B$4:$B$60,$E8)</f>
+        <f>COUNTIF(Control_Plantillas!$B$4:$B$59,$E8)</f>
         <v>2</v>
       </c>
       <c r="G8" s="18">
-        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$60,$E8,Control_Plantillas!$Z$4:$Z$60),0)</f>
+        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$59,$E8,Control_Plantillas!$Z$4:$Z$59),0)</f>
         <v>0.625</v>
       </c>
       <c r="H8" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E8,Control_Plantillas!$I$4:$I$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E8,Control_Plantillas!$I$4:$I$59,"Completado")</f>
         <v>2</v>
       </c>
       <c r="I8" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E8,Control_Plantillas!$L$4:$L$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E8,Control_Plantillas!$L$4:$L$59,"Completado")</f>
         <v>1</v>
       </c>
       <c r="J8" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E8,Control_Plantillas!$O$4:$O$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E8,Control_Plantillas!$O$4:$O$59,"Completado")</f>
         <v>1</v>
       </c>
       <c r="K8" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E8,Control_Plantillas!$R$4:$R$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E8,Control_Plantillas!$R$4:$R$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="L8" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E8,Control_Plantillas!$U$4:$U$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E8,Control_Plantillas!$U$4:$U$59,"Completado")</f>
         <v>0</v>
       </c>
     </row>
@@ -2017,38 +1771,38 @@
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="12">
-        <f>COUNTIF(Control_Plantillas!$I$4:$I$60,"En proceso")</f>
-        <v>32</v>
+        <f>COUNTIF(Control_Plantillas!$I$4:$I$59,"En proceso")</f>
+        <v>31</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>22</v>
       </c>
       <c r="F9" s="17">
-        <f>COUNTIF(Control_Plantillas!$B$4:$B$60,$E9)</f>
+        <f>COUNTIF(Control_Plantillas!$B$4:$B$59,$E9)</f>
         <v>3</v>
       </c>
       <c r="G9" s="18">
-        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$60,$E9,Control_Plantillas!$Z$4:$Z$60),0)</f>
+        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$59,$E9,Control_Plantillas!$Z$4:$Z$59),0)</f>
         <v>0.3</v>
       </c>
       <c r="H9" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E9,Control_Plantillas!$I$4:$I$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E9,Control_Plantillas!$I$4:$I$59,"Completado")</f>
         <v>1</v>
       </c>
       <c r="I9" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E9,Control_Plantillas!$L$4:$L$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E9,Control_Plantillas!$L$4:$L$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="J9" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E9,Control_Plantillas!$O$4:$O$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E9,Control_Plantillas!$O$4:$O$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="K9" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E9,Control_Plantillas!$R$4:$R$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E9,Control_Plantillas!$R$4:$R$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="L9" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E9,Control_Plantillas!$U$4:$U$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E9,Control_Plantillas!$U$4:$U$59,"Completado")</f>
         <v>0</v>
       </c>
     </row>
@@ -2058,38 +1812,38 @@
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="12">
-        <f>COUNTIF(Control_Plantillas!$I$4:$I$60,"No iniciado")</f>
+        <f>COUNTIF(Control_Plantillas!$I$4:$I$59,"No iniciado")</f>
         <v>3</v>
       </c>
       <c r="E10" s="15" t="s">
         <v>30</v>
       </c>
       <c r="F10" s="17">
-        <f>COUNTIF(Control_Plantillas!$B$4:$B$60,$E10)</f>
+        <f>COUNTIF(Control_Plantillas!$B$4:$B$59,$E10)</f>
         <v>23</v>
       </c>
       <c r="G10" s="18">
-        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$60,$E10,Control_Plantillas!$Z$4:$Z$60),0)</f>
+        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$59,$E10,Control_Plantillas!$Z$4:$Z$59),0)</f>
         <v>0.20000000000000007</v>
       </c>
       <c r="H10" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E10,Control_Plantillas!$I$4:$I$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E10,Control_Plantillas!$I$4:$I$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="I10" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E10,Control_Plantillas!$L$4:$L$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E10,Control_Plantillas!$L$4:$L$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="J10" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E10,Control_Plantillas!$O$4:$O$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E10,Control_Plantillas!$O$4:$O$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="K10" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E10,Control_Plantillas!$R$4:$R$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E10,Control_Plantillas!$R$4:$R$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="L10" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E10,Control_Plantillas!$U$4:$U$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E10,Control_Plantillas!$U$4:$U$59,"Completado")</f>
         <v>0</v>
       </c>
     </row>
@@ -2099,7 +1853,7 @@
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="12">
-        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$60,"Bloqueado")</f>
+        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$59,"Bloqueado")</f>
         <v>0</v>
       </c>
       <c r="E11" s="15" t="s">
@@ -2109,8 +1863,8 @@
         <v>5</v>
       </c>
       <c r="G11" s="18">
-        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$60,$E11,Control_Plantillas!$Z$4:$Z$60),0)</f>
-        <v>0.19999999999999998</v>
+        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$59,$E11,Control_Plantillas!$Z$4:$Z$59),0)</f>
+        <v>0.2</v>
       </c>
       <c r="H11" s="17">
         <v>1</v>
@@ -2122,11 +1876,11 @@
         <v>1</v>
       </c>
       <c r="K11" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E11,Control_Plantillas!$R$4:$R$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E11,Control_Plantillas!$R$4:$R$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="L11" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E11,Control_Plantillas!$U$4:$U$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E11,Control_Plantillas!$U$4:$U$59,"Completado")</f>
         <v>0</v>
       </c>
     </row>
@@ -2136,38 +1890,38 @@
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="12">
-        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$60,"Vencido")</f>
-        <v>33</v>
+        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$59,"Vencido")</f>
+        <v>32</v>
       </c>
       <c r="E12" s="15" t="s">
         <v>38</v>
       </c>
       <c r="F12" s="17">
-        <f>COUNTIF(Control_Plantillas!$B$4:$B$60,$E12)</f>
+        <f>COUNTIF(Control_Plantillas!$B$4:$B$59,$E12)</f>
         <v>3</v>
       </c>
       <c r="G12" s="18">
-        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$60,$E12,Control_Plantillas!$Z$4:$Z$60),0)</f>
+        <f>IFERROR(AVERAGEIF(Control_Plantillas!$B$4:$B$59,$E12,Control_Plantillas!$Z$4:$Z$59),0)</f>
         <v>0</v>
       </c>
       <c r="H12" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E12,Control_Plantillas!$I$4:$I$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E12,Control_Plantillas!$I$4:$I$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="I12" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E12,Control_Plantillas!$L$4:$L$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E12,Control_Plantillas!$L$4:$L$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="J12" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E12,Control_Plantillas!$O$4:$O$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E12,Control_Plantillas!$O$4:$O$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="K12" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E12,Control_Plantillas!$R$4:$R$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E12,Control_Plantillas!$R$4:$R$59,"Completado")</f>
         <v>0</v>
       </c>
       <c r="L12" s="17">
-        <f>COUNTIFS(Control_Plantillas!$B$4:$B$60,$E12,Control_Plantillas!$U$4:$U$60,"Completado")</f>
+        <f>COUNTIFS(Control_Plantillas!$B$4:$B$59,$E12,Control_Plantillas!$U$4:$U$59,"Completado")</f>
         <v>0</v>
       </c>
     </row>
@@ -2177,7 +1931,7 @@
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="12">
-        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$60,"En riesgo")</f>
+        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$59,"En riesgo")</f>
         <v>0</v>
       </c>
       <c r="E13" s="26" t="s">
@@ -2188,8 +1942,8 @@
         <v>42</v>
       </c>
       <c r="G13" s="28">
-        <f>IFERROR(AVERAGE(Control_Plantillas!$Z$4:$Z$60),0)</f>
-        <v>0.27674418604651135</v>
+        <f>IFERROR(AVERAGE(Control_Plantillas!$Z$4:$Z$59),0)</f>
+        <v>0.2785714285714283</v>
       </c>
       <c r="H13" s="27">
         <f t="shared" ref="H13:L13" si="0">SUM(H7:H12)</f>
@@ -2218,7 +1972,7 @@
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="12">
-        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$60,"Sin fecha")</f>
+        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$59,"Sin fecha")</f>
         <v>10</v>
       </c>
     </row>
@@ -2228,7 +1982,7 @@
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="12">
-        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$60,"Cerrado")</f>
+        <f ca="1">COUNTIF(Control_Plantillas!$AC$4:$AC$59,"Cerrado")</f>
         <v>0</v>
       </c>
     </row>
@@ -2255,12 +2009,12 @@
         <v>15</v>
       </c>
       <c r="F20" s="17">
-        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$60,$E20)</f>
-        <v>35</v>
+        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$59,$E20)</f>
+        <v>34</v>
       </c>
       <c r="G20" s="18">
         <f t="shared" ref="G20:G25" si="1">IFERROR($F20/SUM($F$20:$F$25),0)</f>
-        <v>0.81395348837209303</v>
+        <v>0.80952380952380953</v>
       </c>
     </row>
     <row r="21" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2268,12 +2022,12 @@
         <v>20</v>
       </c>
       <c r="F21" s="17">
-        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$60,$E21)</f>
+        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$59,$E21)</f>
         <v>2</v>
       </c>
       <c r="G21" s="18">
         <f t="shared" si="1"/>
-        <v>4.6511627906976744E-2</v>
+        <v>4.7619047619047616E-2</v>
       </c>
     </row>
     <row r="22" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2281,7 +2035,7 @@
         <v>27</v>
       </c>
       <c r="F22" s="17">
-        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$60,$E22)</f>
+        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$59,$E22)</f>
         <v>0</v>
       </c>
       <c r="G22" s="18">
@@ -2294,12 +2048,12 @@
         <v>33</v>
       </c>
       <c r="F23" s="17">
-        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$60,$E23)</f>
+        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$59,$E23)</f>
         <v>6</v>
       </c>
       <c r="G23" s="18">
         <f t="shared" si="1"/>
-        <v>0.13953488372093023</v>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="24" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2307,7 +2061,7 @@
         <v>37</v>
       </c>
       <c r="F24" s="17">
-        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$60,$E24)</f>
+        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$59,$E24)</f>
         <v>0</v>
       </c>
       <c r="G24" s="18">
@@ -2320,7 +2074,7 @@
         <v>40</v>
       </c>
       <c r="F25" s="17">
-        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$60,$E25)</f>
+        <f>COUNTIF(Control_Plantillas!$Y$4:$Y$59,$E25)</f>
         <v>0</v>
       </c>
       <c r="G25" s="18">
@@ -6091,7 +5845,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE1000"/>
+  <dimension ref="A1:AE999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -6350,7 +6104,7 @@
       <c r="V4" s="24"/>
       <c r="W4" s="24"/>
       <c r="X4" s="19">
-        <f t="shared" ref="X4:X46" si="0">IF(OR($U4="Completado",$U4="No aplica"),6,IF(OR($R4="Completado",$R4="No aplica"),5,IF(OR($O4="Completado",$O4="No aplica"),4,IF(OR($L4="Completado",$L4="No aplica"),3,IF(OR($I4="Completado",$I4="No aplica"),2,1)))))</f>
+        <f t="shared" ref="X4:X45" si="0">IF(OR($U4="Completado",$U4="No aplica"),6,IF(OR($R4="Completado",$R4="No aplica"),5,IF(OR($O4="Completado",$O4="No aplica"),4,IF(OR($L4="Completado",$L4="No aplica"),3,IF(OR($I4="Completado",$I4="No aplica"),2,1)))))</f>
         <v>4</v>
       </c>
       <c r="Y4" s="25" t="str">
@@ -6362,15 +6116,15 @@
         <v>0.75</v>
       </c>
       <c r="AA4" s="31" t="str">
-        <f t="shared" ref="AA4:AA46" si="1">IF($X4=6,"",IF(IFERROR(INDEX($I4:$V4,3*$X4-1),0)=0,"",INDEX($I4:$V4,3*$X4-1)))</f>
+        <f t="shared" ref="AA4:AA45" si="1">IF($X4=6,"",IF(IFERROR(INDEX($I4:$V4,3*$X4-1),0)=0,"",INDEX($I4:$V4,3*$X4-1)))</f>
         <v/>
       </c>
       <c r="AB4" s="19" t="str">
-        <f t="shared" ref="AB4:AB46" ca="1" si="2">IF($AA4="","",$AA4-TODAY())</f>
+        <f t="shared" ref="AB4:AB45" ca="1" si="2">IF($AA4="","",$AA4-TODAY())</f>
         <v/>
       </c>
       <c r="AC4" s="19" t="str">
-        <f t="shared" ref="AC4:AC46" si="3">IF($X4=6,"Cerrado",IF(OR($I4="Bloqueado",$L4="Bloqueado",$O4="Bloqueado",$R4="Bloqueado",$U4="Bloqueado"),"Bloqueado",IF($AA4="","Sin fecha",IF($AB4&lt;0,"Vencido",IF($AB4&lt;=7,"En riesgo","En tiempo")))))</f>
+        <f t="shared" ref="AC4:AC45" si="3">IF($X4=6,"Cerrado",IF(OR($I4="Bloqueado",$L4="Bloqueado",$O4="Bloqueado",$R4="Bloqueado",$U4="Bloqueado"),"Bloqueado",IF($AA4="","Sin fecha",IF($AB4&lt;0,"Vencido",IF($AB4&lt;=7,"En riesgo","En tiempo")))))</f>
         <v>Sin fecha</v>
       </c>
       <c r="AD4" s="19" t="s">
@@ -9436,22 +9190,22 @@
         <v>Vencido</v>
       </c>
       <c r="AD40" s="19" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="AE40" s="21"/>
     </row>
     <row r="41" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="19" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B41" s="19" t="s">
         <v>35</v>
       </c>
       <c r="C41" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="D41" s="21" t="s">
         <v>271</v>
-      </c>
-      <c r="D41" s="21" t="s">
-        <v>272</v>
       </c>
       <c r="E41" s="22" t="s">
         <v>36</v>
@@ -9521,55 +9275,45 @@
         <v>Vencido</v>
       </c>
       <c r="AD41" s="19" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="AE41" s="21"/>
     </row>
     <row r="42" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="19" t="s">
+        <v>272</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="B42" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="C42" s="19" t="s">
+      <c r="D42" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="D42" s="21" t="s">
-        <v>275</v>
-      </c>
       <c r="E42" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="F42" s="23" t="s">
-        <v>256</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>167</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
       <c r="H42" s="19" t="s">
         <v>18</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J42" s="24">
-        <v>46274</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="J42" s="24"/>
       <c r="K42" s="24"/>
       <c r="L42" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="M42" s="24">
-        <v>46275</v>
-      </c>
+      <c r="M42" s="24"/>
       <c r="N42" s="24"/>
       <c r="O42" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="P42" s="24">
-        <v>46276</v>
-      </c>
+      <c r="P42" s="24"/>
       <c r="Q42" s="24"/>
       <c r="R42" s="19" t="s">
         <v>10</v>
@@ -9591,24 +9335,24 @@
       </c>
       <c r="Z42" s="29">
         <f t="array" ref="Z42">ROUND(Catalogos!$L$3*IFERROR(INDEX(Cat_Factor,MATCH($I42,Cat_Estatus,0)),0)+Catalogos!$L$4*IFERROR(INDEX(Cat_Factor,MATCH($L42,Cat_Estatus,0)),0)+Catalogos!$L$5*IFERROR(INDEX(Cat_Factor,MATCH($O42,Cat_Estatus,0)),0)+Catalogos!$L$6*IFERROR(INDEX(Cat_Factor,MATCH($R42,Cat_Estatus,0)),0)+Catalogos!$L$7*IFERROR(INDEX(Cat_Factor,MATCH($U42,Cat_Estatus,0)),0),4)</f>
-        <v>0.2</v>
-      </c>
-      <c r="AA42" s="31">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="31" t="str">
         <f t="shared" si="1"/>
-        <v>46274</v>
-      </c>
-      <c r="AB42" s="19">
+        <v/>
+      </c>
+      <c r="AB42" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>-3</v>
+        <v/>
       </c>
       <c r="AC42" s="19" t="str">
-        <f t="shared" ca="1" si="3"/>
-        <v>Vencido</v>
-      </c>
-      <c r="AD42" s="19" t="s">
-        <v>269</v>
-      </c>
-      <c r="AE42" s="21"/>
+        <f t="shared" si="3"/>
+        <v>Sin fecha</v>
+      </c>
+      <c r="AD42" s="19"/>
+      <c r="AE42" s="21" t="s">
+        <v>275</v>
+      </c>
     </row>
     <row r="43" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="19" t="s">
@@ -9682,21 +9426,21 @@
       </c>
       <c r="AD43" s="19"/>
       <c r="AE43" s="21" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="44" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="19" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B44" s="19" t="s">
         <v>38</v>
       </c>
       <c r="C44" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="D44" s="21" t="s">
         <v>281</v>
-      </c>
-      <c r="D44" s="21" t="s">
-        <v>282</v>
       </c>
       <c r="E44" s="22" t="s">
         <v>39</v>
@@ -9757,32 +9501,36 @@
       </c>
       <c r="AD44" s="19"/>
       <c r="AE44" s="21" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="45" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="19" t="s">
+        <v>282</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C45" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="D45" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="B45" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>284</v>
-      </c>
-      <c r="D45" s="21" t="s">
-        <v>285</v>
-      </c>
       <c r="E45" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
+        <v>13</v>
+      </c>
+      <c r="F45" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="G45" s="23" t="s">
+        <v>143</v>
+      </c>
       <c r="H45" s="19" t="s">
         <v>18</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J45" s="24"/>
       <c r="K45" s="24"/>
@@ -9816,7 +9564,7 @@
       </c>
       <c r="Z45" s="29">
         <f t="array" ref="Z45">ROUND(Catalogos!$L$3*IFERROR(INDEX(Cat_Factor,MATCH($I45,Cat_Estatus,0)),0)+Catalogos!$L$4*IFERROR(INDEX(Cat_Factor,MATCH($L45,Cat_Estatus,0)),0)+Catalogos!$L$5*IFERROR(INDEX(Cat_Factor,MATCH($O45,Cat_Estatus,0)),0)+Catalogos!$L$6*IFERROR(INDEX(Cat_Factor,MATCH($R45,Cat_Estatus,0)),0)+Catalogos!$L$7*IFERROR(INDEX(Cat_Factor,MATCH($U45,Cat_Estatus,0)),0),4)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AA45" s="31" t="str">
         <f t="shared" si="1"/>
@@ -9830,91 +9578,22 @@
         <f t="shared" si="3"/>
         <v>Sin fecha</v>
       </c>
-      <c r="AD45" s="19"/>
+      <c r="AD45" s="34">
+        <v>46270</v>
+      </c>
       <c r="AE45" s="21" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="46" spans="1:31" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="B46" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="D46" s="21" t="s">
-        <v>287</v>
-      </c>
-      <c r="E46" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F46" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="G46" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="H46" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="I46" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J46" s="24"/>
-      <c r="K46" s="24"/>
-      <c r="L46" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="M46" s="24"/>
-      <c r="N46" s="24"/>
-      <c r="O46" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="P46" s="24"/>
-      <c r="Q46" s="24"/>
-      <c r="R46" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="S46" s="24"/>
-      <c r="T46" s="24"/>
-      <c r="U46" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="V46" s="24"/>
-      <c r="W46" s="24"/>
-      <c r="X46" s="19">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="Y46" s="25" t="str">
-        <f t="array" ref="Y46">INDEX(Cat_Etapas,$X46)</f>
-        <v>1. Llenado de plantilla</v>
-      </c>
-      <c r="Z46" s="29">
-        <f t="array" ref="Z46">ROUND(Catalogos!$L$3*IFERROR(INDEX(Cat_Factor,MATCH($I46,Cat_Estatus,0)),0)+Catalogos!$L$4*IFERROR(INDEX(Cat_Factor,MATCH($L46,Cat_Estatus,0)),0)+Catalogos!$L$5*IFERROR(INDEX(Cat_Factor,MATCH($O46,Cat_Estatus,0)),0)+Catalogos!$L$6*IFERROR(INDEX(Cat_Factor,MATCH($R46,Cat_Estatus,0)),0)+Catalogos!$L$7*IFERROR(INDEX(Cat_Factor,MATCH($U46,Cat_Estatus,0)),0),4)</f>
-        <v>0.2</v>
-      </c>
-      <c r="AA46" s="31" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="AB46" s="19" t="str">
-        <f t="shared" ca="1" si="2"/>
-        <v/>
-      </c>
-      <c r="AC46" s="19" t="str">
-        <f t="shared" si="3"/>
-        <v>Sin fecha</v>
-      </c>
-      <c r="AD46" s="34">
-        <v>46270</v>
-      </c>
-      <c r="AE46" s="21" t="s">
-        <v>288</v>
-      </c>
+        <v>284</v>
+      </c>
+    </row>
+    <row r="46" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="H46" s="35"/>
+      <c r="I46" s="35"/>
+      <c r="L46" s="35"/>
+      <c r="O46" s="35"/>
+      <c r="R46" s="35"/>
+      <c r="U46" s="35"/>
     </row>
     <row r="47" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="35"/>
@@ -10046,16 +9725,7 @@
       <c r="R59" s="35"/>
       <c r="U59" s="35"/>
     </row>
-    <row r="60" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B60" s="35"/>
-      <c r="E60" s="35"/>
-      <c r="H60" s="35"/>
-      <c r="I60" s="35"/>
-      <c r="L60" s="35"/>
-      <c r="O60" s="35"/>
-      <c r="R60" s="35"/>
-      <c r="U60" s="35"/>
-    </row>
+    <row r="60" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="61" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="62" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="63" spans="2:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -10995,9 +10665,8 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <autoFilter ref="A3:AE45"/>
+  <autoFilter ref="A3:AE44"/>
   <mergeCells count="8">
     <mergeCell ref="A1:AE1"/>
     <mergeCell ref="A2:H2"/>
@@ -11008,152 +10677,67 @@
     <mergeCell ref="U2:W2"/>
     <mergeCell ref="X2:AE2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I4:I1000">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+  <conditionalFormatting sqref="I4:I999 L4:L999 O4:O999 R4:R999 U4:U999">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"Completado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I1000">
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+  <conditionalFormatting sqref="I4:I999 L4:L999 O4:O999 R4:R999 U4:U999">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
       <formula>"En proceso"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I1000">
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="equal">
+  <conditionalFormatting sqref="I4:I999 L4:L999 O4:O999 R4:R999 U4:U999 AC4:AC999">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I1000">
-    <cfRule type="cellIs" dxfId="23" priority="4" operator="equal">
+  <conditionalFormatting sqref="I4:I999 L4:L999 O4:O999 R4:R999 U4:U999">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
       <formula>"No aplica"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L1000">
-    <cfRule type="cellIs" dxfId="22" priority="5" operator="equal">
-      <formula>"Completado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L1000">
-    <cfRule type="cellIs" dxfId="21" priority="6" operator="equal">
-      <formula>"En proceso"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L1000">
-    <cfRule type="cellIs" dxfId="20" priority="7" operator="equal">
-      <formula>"Bloqueado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L1000">
-    <cfRule type="cellIs" dxfId="19" priority="8" operator="equal">
-      <formula>"No aplica"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O4:O1000">
-    <cfRule type="cellIs" dxfId="18" priority="9" operator="equal">
-      <formula>"Completado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O4:O1000">
-    <cfRule type="cellIs" dxfId="17" priority="10" operator="equal">
-      <formula>"En proceso"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O4:O1000">
-    <cfRule type="cellIs" dxfId="16" priority="11" operator="equal">
-      <formula>"Bloqueado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O4:O1000">
-    <cfRule type="cellIs" dxfId="15" priority="12" operator="equal">
-      <formula>"No aplica"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R4:R1000">
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="equal">
-      <formula>"Completado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R4:R1000">
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
-      <formula>"En proceso"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R4:R1000">
-    <cfRule type="cellIs" dxfId="12" priority="15" operator="equal">
-      <formula>"Bloqueado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R4:R1000">
-    <cfRule type="cellIs" dxfId="11" priority="16" operator="equal">
-      <formula>"No aplica"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U4:U1000">
-    <cfRule type="cellIs" dxfId="10" priority="17" operator="equal">
-      <formula>"Completado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U4:U1000">
-    <cfRule type="cellIs" dxfId="9" priority="18" operator="equal">
-      <formula>"En proceso"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U4:U1000">
-    <cfRule type="cellIs" dxfId="8" priority="19" operator="equal">
-      <formula>"Bloqueado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U4:U1000">
-    <cfRule type="cellIs" dxfId="7" priority="20" operator="equal">
-      <formula>"No aplica"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB4:AB1000">
-    <cfRule type="cellIs" dxfId="6" priority="21" operator="lessThan">
+  <conditionalFormatting sqref="AB4:AB999">
+    <cfRule type="cellIs" dxfId="5" priority="21" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC1000">
-    <cfRule type="cellIs" dxfId="5" priority="22" operator="equal">
+  <conditionalFormatting sqref="AC4:AC999">
+    <cfRule type="cellIs" dxfId="4" priority="22" operator="equal">
       <formula>"Cerrado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC1000">
-    <cfRule type="cellIs" dxfId="4" priority="23" operator="equal">
+  <conditionalFormatting sqref="AC4:AC999">
+    <cfRule type="cellIs" dxfId="3" priority="23" operator="equal">
       <formula>"En tiempo"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC1000">
-    <cfRule type="cellIs" dxfId="3" priority="24" operator="equal">
+  <conditionalFormatting sqref="AC4:AC999">
+    <cfRule type="cellIs" dxfId="2" priority="24" operator="equal">
       <formula>"En riesgo"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC1000">
-    <cfRule type="cellIs" dxfId="2" priority="25" operator="equal">
+  <conditionalFormatting sqref="AC4:AC999">
+    <cfRule type="cellIs" dxfId="1" priority="25" operator="equal">
       <formula>"Vencido"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC1000">
-    <cfRule type="cellIs" dxfId="1" priority="26" operator="equal">
-      <formula>"Bloqueado"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC4:AC1000">
+  <conditionalFormatting sqref="AC4:AC999">
     <cfRule type="cellIs" dxfId="0" priority="27" operator="equal">
       <formula>"Sin fecha"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="H4:H60">
+    <dataValidation type="list" allowBlank="1" sqref="H4:H59">
       <formula1>Cat_Prioridad</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I4:I60 L4:L60 O4:O60 R4:R60 U4:U60">
+    <dataValidation type="list" allowBlank="1" sqref="U4:U59 R4:R59 O4:O59 L4:L59 I4:I59">
       <formula1>Cat_Estatus</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E4:E60">
+    <dataValidation type="list" allowBlank="1" sqref="E4:E59">
       <formula1>Cat_Areas</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B4:B60">
+    <dataValidation type="list" allowBlank="1" sqref="B4:B59">
       <formula1>Cat_Modulos</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>